<commit_message>
Three official checklist packs from controlled forms: VAC-001 vendor (25, replaces draft), SAC-001 school safety SMS (26, dual Doc/Impl), SSC-001 surveillance spot check (29); docx->pack converter; Portal back button in all apps; restore template.html from HEAD after accidental overwrite with old version
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/packs/vendor/v2026/checklist.xlsx
+++ b/packs/vendor/v2026/checklist.xlsx
@@ -423,27 +423,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
-    <col width="50" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="50" customWidth="1" min="16" max="16"/>
-    <col width="7" customWidth="1" min="17" max="17"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -528,6 +509,11 @@
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
+          <t>SubChecklist</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>Dual</t>
         </is>
       </c>
@@ -540,27 +526,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Vendor / Contracted Activities Audit</t>
+          <t>Vendor / Contracted Services Audit</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>การตรวจผู้ให้บริการภายนอก/กิจกรรมจ้างช่วง</t>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>สัญญาจ้าง + OMM Section 5 (Compliance Monitoring)</t>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Part 1 – Contract &amp; Oversight</t>
+          <t>V1 – Contract, Approvals &amp; Insurance</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>สัญญาและการกำกับดูแลการจ้างช่วง</t>
+          <t>สัญญา การรับรอง และประกันภัย</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -571,37 +557,34 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Contract documentation</t>
+          <t>V1.1  Contract status / สถานะสัญญา</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>A written contract/agreement exists for each contracted activity, defining scope of work, standards and responsibilities.</t>
+          <t>A written contract/SLA exists, is current, and its scope matches the services actually being provided to the ATO.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>มีสัญญา/ข้อตกลงเป็นลายลักษณ์อักษรสำหรับทุกกิจกรรมที่จ้างช่วง ระบุขอบเขตงาน มาตรฐาน และความรับผิดชอบ</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>ORA.GEN.205</t>
-        </is>
-      </c>
+          <t>มีสัญญา/ข้อตกลงเป็นลายลักษณ์อักษร ยังมีผล และขอบเขตตรงกับบริการที่ให้จริง</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
-          <t>แฟ้มสัญญา / PO</t>
+          <t>OMM contracted activities list</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>ตรวจแฟ้มสัญญาทุกราย: ขอบเขตงาน มาตรฐานอ้างอิง ผู้รับผิดชอบ วันเริ่ม-สิ้นสุด ลายเซ็นครบ</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
+          <t>ตรวจบันทึก / ตรวจไขว้</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -615,27 +598,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Vendor / Contracted Activities Audit</t>
+          <t>Vendor / Contracted Services Audit</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>การตรวจผู้ให้บริการภายนอก/กิจกรรมจ้างช่วง</t>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>สัญญาจ้าง + OMM Section 5 (Compliance Monitoring)</t>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Part 1 – Contract &amp; Oversight</t>
+          <t>V1 – Contract, Approvals &amp; Insurance</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>สัญญาและการกำกับดูแลการจ้างช่วง</t>
+          <t>สัญญา การรับรอง และประกันภัย</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -646,37 +629,34 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Contract documentation</t>
+          <t>V1.1  Contract status / สถานะสัญญา</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>The contract states that the ATO retains responsibility for the contracted activity and ensures compliance with applicable requirements.</t>
+          <t>The vendor holds all certificates/approvals required for the service (e.g. AMO approval, fuel supplier authorisation, aerodrome licence, exam/medical provider approval) and they are current.</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>สัญญาระบุว่า ATO ยังคงเป็นผู้รับผิดชอบต่อกิจกรรมที่จ้างช่วง และกำกับให้เป็นไปตามข้อกำหนดที่เกี่ยวข้อง</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>ORA.GEN.205</t>
-        </is>
-      </c>
+          <t>ผู้ให้บริการมีใบรับรอง/การอนุมัติที่จำเป็นครบและยังไม่หมดอายุ (เช่น AMO approval, ใบอนุญาตสนามบิน, การรับรองผู้ให้บริการสอบ/แพทย์)</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
-          <t>ข้อความในสัญญา</t>
+          <t>Vendor certificates file</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>อ่านข้อสัญญา: มี clause ความรับผิดชอบของ ATO และสิทธิเข้าตรวจสอบ (right of audit)</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
+          <t>ตรวจบันทึก</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -690,68 +670,65 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Vendor / Contracted Activities Audit</t>
+          <t>Vendor / Contracted Services Audit</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>การตรวจผู้ให้บริการภายนอก/กิจกรรมจ้างช่วง</t>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>สัญญาจ้าง + OMM Section 5 (Compliance Monitoring)</t>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Part 1 – Contract &amp; Oversight</t>
+          <t>V1 – Contract, Approvals &amp; Insurance</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>สัญญาและการกำกับดูแลการจ้างช่วง</t>
+          <t>สัญญา การรับรอง และประกันภัย</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Vendor register</t>
+          <t>V1.1  Contract status / สถานะสัญญา</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>A current register of all vendors/contracted activities is maintained with status and review dates.</t>
+          <t>Vendor liability insurance is valid and adequate for the service provided.</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>มีทะเบียนผู้ให้บริการ/กิจกรรมจ้างช่วงเป็นปัจจุบัน พร้อมสถานะและวันทบทวน</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>OMM Section 5</t>
-        </is>
-      </c>
+          <t>ประกันภัยความรับผิดของผู้ให้บริการยังมีผลและวงเงินเพียงพอ</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr">
         <is>
-          <t>ทะเบียน Vendor</t>
+          <t>Insurance certificate</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>เทียบทะเบียนกับสัญญาจริง: ครบทุกราย วันทบทวนไม่หมดอายุ</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
+          <t>ตรวจบันทึก</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -765,68 +742,65 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Vendor / Contracted Activities Audit</t>
+          <t>Vendor / Contracted Services Audit</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>การตรวจผู้ให้บริการภายนอก/กิจกรรมจ้างช่วง</t>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>สัญญาจ้าง + OMM Section 5 (Compliance Monitoring)</t>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Part 1 – Contract &amp; Oversight</t>
+          <t>V1 – Contract, Approvals &amp; Insurance</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>สัญญาและการกำกับดูแลการจ้างช่วง</t>
+          <t>สัญญา การรับรอง และประกันภัย</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Vendor register</t>
+          <t>V1.1  Contract status / สถานะสัญญา</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Contracted activities are included in the ATO compliance monitoring (audit) programme.</t>
+          <t>Any subcontracting by the vendor is disclosed and acceptable to the ATO.</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>กิจกรรมจ้างช่วงถูกรวมอยู่ในแผนการตรวจติดตามภายใน (audit programme) ของ ATO</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>ORA.GEN.200(a)(6)</t>
-        </is>
-      </c>
+          <t>การจ้างช่วงต่อ (ถ้ามี) ได้แจ้งให้ ATO ทราบและยอมรับได้</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Audit Plan ประจำปี</t>
+          <t>Contract subcontracting clause</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>เปิด Audit Plan: มีรายการตรวจ vendor อย่างน้อยตามรอบที่กำหนด</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
+          <t>ตรวจบันทึก / สัมภาษณ์</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -840,27 +814,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Vendor / Contracted Activities Audit</t>
+          <t>Vendor / Contracted Services Audit</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>การตรวจผู้ให้บริการภายนอก/กิจกรรมจ้างช่วง</t>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>สัญญาจ้าง + OMM Section 5 (Compliance Monitoring)</t>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Part 2 – Vendor Qualification</t>
+          <t>V2 – Organisation &amp; Personnel Competence</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>คุณสมบัติและการรับรองของผู้ให้บริการ</t>
+          <t>องค์กรและความสามารถของบุคลากร</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -871,37 +845,34 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Approvals &amp; certificates</t>
+          <t>V2.1  Personnel / บุคลากรผู้ให้บริการ</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>The vendor holds valid approvals/certificates/licences required for the contracted activity.</t>
+          <t>Personnel performing the service hold the required licences/qualifications; records sighted (e.g. maintenance personnel licences, fuel handler training, instructor/examiner approvals).</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>ผู้ให้บริการมีใบรับรอง/ใบอนุญาตที่จำเป็นสำหรับงานที่จ้าง และยังไม่หมดอายุ</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>ORA.GEN.205</t>
-        </is>
-      </c>
+          <t>บุคลากรที่ปฏิบัติงานมีใบอนุญาต/คุณสมบัติตามที่กำหนด และตรวจเห็นบันทึกจริง</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr">
         <is>
-          <t>สำเนาใบรับรอง</t>
+          <t>Vendor personnel files</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>ตรวจสำเนาใบรับรอง: ขอบเขตครอบคลุมงานที่จ้าง วันหมดอายุ มีระบบเตือนต่ออายุ</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
+          <t>ตรวจบันทึก</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -915,27 +886,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Vendor / Contracted Activities Audit</t>
+          <t>Vendor / Contracted Services Audit</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>การตรวจผู้ให้บริการภายนอก/กิจกรรมจ้างช่วง</t>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>สัญญาจ้าง + OMM Section 5 (Compliance Monitoring)</t>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Part 2 – Vendor Qualification</t>
+          <t>V2 – Organisation &amp; Personnel Competence</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>คุณสมบัติและการรับรองของผู้ให้บริการ</t>
+          <t>องค์กรและความสามารถของบุคลากร</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -946,37 +917,30 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Approvals &amp; certificates</t>
+          <t>V2.1  Personnel / บุคลากรผู้ให้บริการ</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Personnel of the vendor performing the activity are qualified and their qualifications are on record.</t>
+          <t>Recurrent/refresher training of vendor personnel is current where required (e.g. dangerous goods, fuel quality control, human factors for AMO staff).</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>บุคลากรของผู้ให้บริการที่ปฏิบัติงานมีคุณสมบัติครบ และมีหลักฐานคุณสมบัติเก็บไว้</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>ORA.GEN.205</t>
-        </is>
-      </c>
+          <t>การอบรมทบทวนของบุคลากรผู้ให้บริการเป็นปัจจุบันตามที่กำหนด</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>แฟ้มประวัติบุคลากร vendor</t>
-        </is>
-      </c>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>สุ่มตรวจรายชื่อผู้ปฏิบัติงานจริงเทียบแฟ้มคุณสมบัติ/ใบอนุญาต</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
+          <t>ตรวจบันทึก</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -990,68 +954,61 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Vendor / Contracted Activities Audit</t>
+          <t>Vendor / Contracted Services Audit</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>การตรวจผู้ให้บริการภายนอก/กิจกรรมจ้างช่วง</t>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>สัญญาจ้าง + OMM Section 5 (Compliance Monitoring)</t>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Part 2 – Vendor Qualification</t>
+          <t>V2 – Organisation &amp; Personnel Competence</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>คุณสมบัติและการรับรองของผู้ให้บริการ</t>
+          <t>องค์กรและความสามารถของบุคลากร</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Initial evaluation</t>
+          <t>V2.1  Personnel / บุคลากรผู้ให้บริการ</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>An initial evaluation of the vendor was performed and documented before contract award.</t>
+          <t>Staffing level is adequate for the service demand; a named contact and escalation route for the ATO exists.</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>มีการประเมินผู้ให้บริการก่อนทำสัญญา และบันทึกผลไว้</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>OMM Section 5</t>
-        </is>
-      </c>
+          <t>อัตรากำลังเพียงพอต่อปริมาณงาน มีผู้ประสานงานหลักและช่องทางยกระดับปัญหา</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>แบบประเมินก่อนจ้าง</t>
-        </is>
-      </c>
+      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>ดูบันทึกการประเมินครั้งแรก: เกณฑ์ ผลประเมิน ผู้อนุมัติ</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
+          <t>สัมภาษณ์</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1065,27 +1022,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Vendor / Contracted Activities Audit</t>
+          <t>Vendor / Contracted Services Audit</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>การตรวจผู้ให้บริการภายนอก/กิจกรรมจ้างช่วง</t>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>สัญญาจ้าง + OMM Section 5 (Compliance Monitoring)</t>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Part 3 – Service Delivery &amp; Quality</t>
+          <t>V3 – Facilities &amp; Equipment</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>การส่งมอบงานและคุณภาพ</t>
+          <t>สถานที่และอุปกรณ์ของผู้ให้บริการ</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1096,37 +1053,30 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Service performance</t>
+          <t>V3.1  Facilities &amp; equipment / สิ่งอำนวยความสะดวก</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Services are delivered in accordance with the contract and applicable manuals/procedures of the ATO.</t>
+          <t>Facilities and equipment used for the service are adequate, serviceable and maintained (storage tanks, workshop, test equipment, classrooms as applicable).</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>การส่งมอบงานเป็นไปตามสัญญาและสอดคล้องกับคู่มือ/ขั้นตอนของ ATO</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>ORA.GEN.205</t>
-        </is>
-      </c>
+          <t>สถานที่และอุปกรณ์เพียงพอ ใช้งานได้ และได้รับการบำรุงรักษา</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>บันทึกรับมอบงาน</t>
-        </is>
-      </c>
+      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t>สุ่มตรวจงานที่ส่งมอบล่าสุดเทียบข้อกำหนดในสัญญาและคู่มือที่เกี่ยวข้อง</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
+          <t>สังเกตการณ์</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1140,27 +1090,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Vendor / Contracted Activities Audit</t>
+          <t>Vendor / Contracted Services Audit</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>การตรวจผู้ให้บริการภายนอก/กิจกรรมจ้างช่วง</t>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>สัญญาจ้าง + OMM Section 5 (Compliance Monitoring)</t>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Part 3 – Service Delivery &amp; Quality</t>
+          <t>V3 – Facilities &amp; Equipment</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>การส่งมอบงานและคุณภาพ</t>
+          <t>สถานที่และอุปกรณ์ของผู้ให้บริการ</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1171,37 +1121,30 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Service performance</t>
+          <t>V3.1  Facilities &amp; equipment / สิ่งอำนวยความสะดวก</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Nonconformities in vendor services are recorded and corrective action is requested and followed up (CAR).</t>
+          <t>Measuring/test equipment is calibrated and within calibration due dates (torque wrenches, fuel test kits, pressure gauges).</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>ข้อบกพร่องจากงานของผู้ให้บริการถูกบันทึก ออก CAR และติดตามจนปิด</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>OMM Section 5</t>
-        </is>
-      </c>
+          <t>เครื่องมือวัด/ทดสอบผ่านการสอบเทียบและยังไม่เกินกำหนด</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>ทะเบียน CAR</t>
-        </is>
-      </c>
+      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
-          <t>ตรวจทะเบียน CAR ที่เกี่ยวกับ vendor: ตอบกลับตามกำหนด ปิดโดยมีหลักฐานทวนสอบ</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
+          <t>ตรวจบันทึก / สังเกตการณ์</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1215,68 +1158,61 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Vendor / Contracted Activities Audit</t>
+          <t>Vendor / Contracted Services Audit</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>การตรวจผู้ให้บริการภายนอก/กิจกรรมจ้างช่วง</t>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>สัญญาจ้าง + OMM Section 5 (Compliance Monitoring)</t>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Part 3 – Service Delivery &amp; Quality</t>
+          <t>V3 – Facilities &amp; Equipment</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>การส่งมอบงานและคุณภาพ</t>
+          <t>สถานที่และอุปกรณ์ของผู้ให้บริการ</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Periodic review</t>
+          <t>V3.1  Facilities &amp; equipment / สิ่งอำนวยความสะดวก</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Vendor performance is reviewed periodically and results feed the management review.</t>
+          <t>Safety equipment at vendor facility is serviceable (fire extinguishers in date, spill kits, PPE available and used).</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>มีการทบทวนผลงานผู้ให้บริการตามรอบ และนำผลเข้าประชุมทบทวนฝ่ายบริหาร</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>ORA.GEN.200(a)(5)</t>
-        </is>
-      </c>
+          <t>อุปกรณ์ความปลอดภัย ณ สถานที่ผู้ให้บริการพร้อมใช้ (ถังดับเพลิง, ชุดจัดการหกรั่วไหล, PPE)</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>รายงานประชุมทบทวน</t>
-        </is>
-      </c>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>ดูรายงาน management review ล่าสุด: มีวาระผลงาน vendor</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
+          <t>สังเกตการณ์</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1290,27 +1226,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Vendor / Contracted Activities Audit</t>
+          <t>Vendor / Contracted Services Audit</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>การตรวจผู้ให้บริการภายนอก/กิจกรรมจ้างช่วง</t>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>สัญญาจ้าง + OMM Section 5 (Compliance Monitoring)</t>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Part 4 – Safety &amp; SMS Interface</t>
+          <t>V4 – Service Delivery by Type</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ความปลอดภัยและการเชื่อมต่อ SMS</t>
+          <t>การส่งมอบบริการตามประเภท (ข้ามส่วนที่ไม่เกี่ยวข้อง = N/A)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1321,37 +1257,34 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Hazard &amp; occurrence reporting</t>
+          <t>V4.1  Fuel services / บริการเชื้อเพลิง (If applicable)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>The vendor is included in the ATO hazard/occurrence reporting system and knows how to report.</t>
+          <t>Fuel grade supplied is correct for the fleet; storage and dispensing quality control performed and recorded (daily water checks, filter checks, sampling).</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>ผู้ให้บริการอยู่ในระบบรายงานอันตราย/เหตุการณ์ของ ATO และทราบช่องทางการรายงาน</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>ORA.GEN.200(a)(3)</t>
-        </is>
-      </c>
+          <t>เกรดเชื้อเพลิงถูกต้องกับฝูงบิน มีการควบคุมคุณภาพการจัดเก็บ/จ่าย และบันทึกจริง (ตรวจน้ำประจำวัน ตรวจไส้กรอง เก็บตัวอย่าง)</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr">
         <is>
-          <t>บันทึกรายงาน/การสื่อสาร</t>
+          <t>Fuel QC log</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>สัมภาษณ์ผู้ปฏิบัติงาน vendor: ทราบช่องทางรายงาน · ดูตัวอย่างรายงานที่เคยส่ง</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
+          <t>ตรวจบันทึก / สังเกตการณ์</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1365,27 +1298,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Vendor / Contracted Activities Audit</t>
+          <t>Vendor / Contracted Services Audit</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>การตรวจผู้ให้บริการภายนอก/กิจกรรมจ้างช่วง</t>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>สัญญาจ้าง + OMM Section 5 (Compliance Monitoring)</t>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Part 4 – Safety &amp; SMS Interface</t>
+          <t>V4 – Service Delivery by Type</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>ความปลอดภัยและการเชื่อมต่อ SMS</t>
+          <t>การส่งมอบบริการตามประเภท (ข้ามส่วนที่ไม่เกี่ยวข้อง = N/A)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -1396,37 +1329,30 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Hazard &amp; occurrence reporting</t>
+          <t>V4.1  Fuel services / บริการเชื้อเพลิง (If applicable)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Safety-relevant changes at the vendor (personnel, equipment, procedures) are communicated to the ATO (management of change).</t>
+          <t>Refuelling practice observed complies with fire precautions: bonding, extinguisher positioned, no occupants during fuelling, spill procedure known.</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>การเปลี่ยนแปลงที่กระทบความปลอดภัยฝั่งผู้ให้บริการ (คน/อุปกรณ์/ขั้นตอน) ถูกแจ้งให้ ATO ทราบ</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>ORA.GEN.130</t>
-        </is>
-      </c>
+          <t>การเติมเชื้อเพลิงที่สังเกตเป็นไปตามข้อควรระวังอัคคีภัย</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>บันทึก MOC</t>
-        </is>
-      </c>
+      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
-          <t>ดูหลักฐานการแจ้งการเปลี่ยนแปลงล่าสุด และการประเมินผลกระทบโดย ATO</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
+          <t>สังเกตการณ์ / สัมภาษณ์</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1440,68 +1366,885 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Vendor / Contracted Activities Audit</t>
+          <t>Vendor / Contracted Services Audit</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>การตรวจผู้ให้บริการภายนอก/กิจกรรมจ้างช่วง</t>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>สัญญาจ้าง + OMM Section 5 (Compliance Monitoring)</t>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Part 4 – Safety &amp; SMS Interface</t>
+          <t>V4 – Service Delivery by Type</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>ความปลอดภัยและการเชื่อมต่อ SMS</t>
+          <t>การส่งมอบบริการตามประเภท (ข้ามส่วนที่ไม่เกี่ยวข้อง = N/A)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Emergency &amp; contingency</t>
+          <t>V4.1  Fuel services / บริการเชื้อเพลิง (If applicable)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Contingency arrangements exist for interruption of the contracted service.</t>
+          <t>Fuel uplift documentation is accurate and traceable to aircraft and payment records.</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>มีแผนรองรับกรณีผู้ให้บริการหยุดให้บริการ/ส่งมอบไม่ได้</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>OMM Section 3</t>
-        </is>
-      </c>
+          <t>เอกสารการเติมเชื้อเพลิงถูกต้อง ตรวจสอบย้อนถึงอากาศยานและบันทึกการชำระได้</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>แผน contingency</t>
-        </is>
-      </c>
+      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
-          <t>ดูแผนสำรอง: ระบุทางเลือก ผู้รับผิดชอบ และเคยทบทวนเมื่อใด</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
+          <t>ตรวจไขว้</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>VEN</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Vendor / Contracted Services Audit</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>V4 – Service Delivery by Type</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>การส่งมอบบริการตามประเภท (ข้ามส่วนที่ไม่เกี่ยวข้อง = N/A)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>V4.2  Maintenance / AMO (If applicable)</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Work is performed under work orders using current approved maintenance data; CRS issued by authorised certifying staff after each maintenance event.</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>งานซ่อมทำตาม work order โดยใช้ maintenance data ฉบับปัจจุบัน และออก CRS โดยผู้มีอำนาจทุกครั้ง</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>MMSOP Work Order / AMO procedures</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>ตรวจบันทึก / ตรวจไขว้</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>VEN</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Vendor / Contracted Services Audit</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>V4 – Service Delivery by Type</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>การส่งมอบบริการตามประเภท (ข้ามส่วนที่ไม่เกี่ยวข้อง = N/A)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>V4.2  Maintenance / AMO (If applicable)</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Parts and materials are traceable (release certificates / batch numbers); unserviceable parts segregated and tagged.</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>อะไหล่/วัสดุตรวจสอบย้อนได้ (ใบรับรอง/หมายเลข batch) ชิ้นส่วนใช้ไม่ได้แยกเก็บและติดป้าย</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>ตรวจบันทึก / สังเกตการณ์</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>VEN</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Vendor / Contracted Services Audit</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>V4 – Service Delivery by Type</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>การส่งมอบบริการตามประเภท (ข้ามส่วนที่ไม่เกี่ยวข้อง = N/A)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>V4.2  Maintenance / AMO (If applicable)</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Tool control is practised (tool accountability check before/after work, calibrated tools in date).</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>มีการควบคุมเครื่องมือจริง (นับก่อน-หลังงาน, เครื่องมือสอบเทียบไม่หมดอายุ)</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>MMSOP Tool Accountability</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>สังเกตการณ์</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>VEN</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Vendor / Contracted Services Audit</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>V4 – Service Delivery by Type</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>การส่งมอบบริการตามประเภท (ข้ามส่วนที่ไม่เกี่ยวข้อง = N/A)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>V4.2  Maintenance / AMO (If applicable)</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Defects deferred by the AMO follow the agreed procedure/MEL and are communicated to the ATO before flight.</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>ข้อบกพร่องที่ defer ทำตามขั้นตอน/MEL และแจ้ง ATO ก่อนทำการบิน</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>ตรวจบันทึก / สัมภาษณ์</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>VEN</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Vendor / Contracted Services Audit</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>V4 – Service Delivery by Type</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>การส่งมอบบริการตามประเภท (ข้ามส่วนที่ไม่เกี่ยวข้อง = N/A)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>V4.3  Aerodrome services / บริการสนามบิน (If applicable)</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Runway/movement area inspections are performed per schedule; defects/NOTAM initiated when required.</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>การตรวจทางวิ่ง/พื้นที่เคลื่อนไหวทำตามวาระ และออก NOTAM เมื่อจำเป็น</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>ตรวจบันทึก / สัมภาษณ์</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>VEN</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Vendor / Contracted Services Audit</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>V4 – Service Delivery by Type</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>การส่งมอบบริการตามประเภท (ข้ามส่วนที่ไม่เกี่ยวข้อง = N/A)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>V4.3  Aerodrome services / บริการสนามบิน (If applicable)</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Rescue &amp; firefighting capability and wildlife hazard control are maintained as agreed.</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>ขีดความสามารถกู้ภัยดับเพลิงและการควบคุมสัตว์อันตรายคงอยู่ตามข้อตกลง</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>สังเกตการณ์ / ตรวจบันทึก</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>VEN</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Vendor / Contracted Services Audit</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>V4 – Service Delivery by Type</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>การส่งมอบบริการตามประเภท (ข้ามส่วนที่ไม่เกี่ยวข้อง = N/A)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>V4.4  Training / examination / medical services (If applicable)</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>External training/exam/medical services hold current approvals and deliver records back to the ATO in the agreed format and time.</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>บริการอบรม/สอบ/แพทย์ภายนอกมีการรับรองปัจจุบัน และส่งบันทึกผลกลับให้ ATO ตามรูปแบบ/เวลาที่ตกลง</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>ตรวจบันทึก / ตรวจไขว้</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>VEN</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Vendor / Contracted Services Audit</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>V5 – Safety &amp; Quality Interface</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>จุดเชื่อมต่อด้านนิรภัยและคุณภาพกับ ATO</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>V5.1  Interface / การเชื่อมโยงระบบ</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Occurrences/hazards detected by the vendor that affect the ATO are reported to the ATO safety system (evidence of at least the channel being known).</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>เหตุการณ์/อันตรายที่ผู้ให้บริการพบและกระทบ ATO ถูกส่งเข้าระบบนิรภัยของ ATO (อย่างน้อยรู้ช่องทาง)</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>สัมภาษณ์ / ตรวจบันทึก</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>VEN</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Vendor / Contracted Services Audit</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>V5 – Safety &amp; Quality Interface</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>จุดเชื่อมต่อด้านนิรภัยและคุณภาพกับ ATO</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>V5.1  Interface / การเชื่อมโยงระบบ</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>The vendor has its own internal QA/inspection for the service, and results are available to the ATO on request.</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>ผู้ให้บริการมีการตรวจสอบคุณภาพภายในของตนเอง และ ATO ขอดูผลได้</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>ตรวจบันทึก</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>VEN</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Vendor / Contracted Services Audit</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>V5 – Safety &amp; Quality Interface</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>จุดเชื่อมต่อด้านนิรภัยและคุณภาพกับ ATO</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>V5.1  Interface / การเชื่อมโยงระบบ</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Findings from previous ATO vendor audits are closed with evidence.</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>ข้อบกพร่องจากการตรวจผู้ให้บริการครั้งก่อนปิดแล้วพร้อมหลักฐาน</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>ตรวจบันทึก</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>VEN</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Vendor / Contracted Services Audit</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>V6 – Records &amp; Performance Monitoring</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>บันทึกและการติดตามผลการให้บริการ</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>V6.1  Performance / ผลการให้บริการ</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Service records delivered to the ATO are complete and retained per the ATO record-keeping requirements.</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>บันทึกการให้บริการที่ส่งให้ ATO ครบถ้วนและถูกจัดเก็บตามข้อกำหนดการเก็บบันทึกของ ATO</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>ตรวจบันทึก</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>VEN</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Vendor / Contracted Services Audit</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>การตรวจผู้ให้บริการภายนอก</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>D-0507-VAC-001 · ORA.GEN.205 · OMM Section 5</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>V6 – Records &amp; Performance Monitoring</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>บันทึกและการติดตามผลการให้บริการ</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>V6.1  Performance / ผลการให้บริการ</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Service performance is monitored (delays, defect recurrence, complaints) and reviewed with the vendor; corrective actions agreed where needed.</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>มีการติดตามผลการให้บริการ (ความล่าช้า ข้อบกพร่องซ้ำ ข้อร้องเรียน) และทบทวนร่วมกับผู้ให้บริการ</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>ตรวจบันทึก / สัมภาษณ์</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>